<commit_message>
more bug fixes + data cleanup
</commit_message>
<xml_diff>
--- a/FoodBank Files/Product In.xlsx
+++ b/FoodBank Files/Product In.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\icarusjay\Downloads\xampp\htdocs\FoodBank Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F155499-66E5-4F37-8F88-7A515966A58B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E3459C4-2004-4A92-965F-730AF53B9A12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13740" xr2:uid="{FEF8D386-D128-4069-BDCD-FE457B1D9085}"/>
   </bookViews>
@@ -62,9 +62,6 @@
     <t>PACKED BY</t>
   </si>
   <si>
-    <t>TOTAL COST(₱)</t>
-  </si>
-  <si>
     <t>EXPIRY DATE</t>
   </si>
   <si>
@@ -576,6 +573,9 @@
   </si>
   <si>
     <t>WEIGHT(KG)</t>
+  </si>
+  <si>
+    <t>COST</t>
   </si>
 </sst>
 </file>
@@ -1011,42 +1011,42 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
         <v>14</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>15</v>
-      </c>
-      <c r="F2" t="s">
-        <v>16</v>
       </c>
       <c r="G2">
         <v>2</v>
       </c>
       <c r="H2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I2">
         <v>0.33</v>
@@ -1055,36 +1055,36 @@
         <v>0</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G3">
         <v>3</v>
       </c>
       <c r="H3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I3">
         <v>0.33</v>
@@ -1093,36 +1093,36 @@
         <v>0</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" t="s">
         <v>22</v>
-      </c>
-      <c r="F4" t="s">
-        <v>23</v>
       </c>
       <c r="G4">
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I4">
         <v>0.35</v>
@@ -1131,36 +1131,36 @@
         <v>0</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="L4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G5">
         <v>1</v>
       </c>
       <c r="H5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I5">
         <v>0.35</v>
@@ -1169,36 +1169,36 @@
         <v>0</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G6">
         <v>1</v>
       </c>
       <c r="H6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I6">
         <v>0.35</v>
@@ -1207,36 +1207,36 @@
         <v>0</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G7">
         <v>3</v>
       </c>
       <c r="H7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I7">
         <v>0.28000000000000003</v>
@@ -1245,36 +1245,36 @@
         <v>0</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="L7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G8">
         <v>3</v>
       </c>
       <c r="H8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I8">
         <v>0.33</v>
@@ -1283,36 +1283,36 @@
         <v>0</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G9">
         <v>7</v>
       </c>
       <c r="H9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I9">
         <v>0.33</v>
@@ -1321,36 +1321,36 @@
         <v>0</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G10">
         <v>2</v>
       </c>
       <c r="H10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I10">
         <v>0.33</v>
@@ -1359,36 +1359,36 @@
         <v>0</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G11">
         <v>6</v>
       </c>
       <c r="H11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I11">
         <v>0.18</v>
@@ -1397,36 +1397,36 @@
         <v>0</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G12">
         <v>27</v>
       </c>
       <c r="H12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I12">
         <v>0.34</v>
@@ -1435,36 +1435,36 @@
         <v>0</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G13">
         <v>44</v>
       </c>
       <c r="H13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I13">
         <v>0.36</v>
@@ -1473,36 +1473,36 @@
         <v>0</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="L13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E14" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" t="s">
         <v>39</v>
-      </c>
-      <c r="F14" t="s">
-        <v>40</v>
       </c>
       <c r="G14">
         <v>1</v>
       </c>
       <c r="H14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I14">
         <v>0.22</v>
@@ -1511,36 +1511,36 @@
         <v>0</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E15" t="s">
+        <v>42</v>
+      </c>
+      <c r="F15" t="s">
         <v>43</v>
-      </c>
-      <c r="F15" t="s">
-        <v>44</v>
       </c>
       <c r="G15">
         <v>1</v>
       </c>
       <c r="H15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I15">
         <v>0.12</v>
@@ -1549,36 +1549,36 @@
         <v>0</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="L15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E16" t="s">
+        <v>44</v>
+      </c>
+      <c r="F16" t="s">
         <v>45</v>
-      </c>
-      <c r="F16" t="s">
-        <v>46</v>
       </c>
       <c r="G16">
         <v>4</v>
       </c>
       <c r="H16" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I16">
         <v>0.24</v>
@@ -1587,36 +1587,36 @@
         <v>0</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D17" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G17">
         <v>1</v>
       </c>
       <c r="H17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I17">
         <v>0.5</v>
@@ -1625,36 +1625,36 @@
         <v>0</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="L17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E18" t="s">
+        <v>50</v>
+      </c>
+      <c r="F18" t="s">
         <v>51</v>
-      </c>
-      <c r="F18" t="s">
-        <v>52</v>
       </c>
       <c r="G18">
         <v>1</v>
       </c>
       <c r="H18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I18">
         <v>0.5</v>
@@ -1663,36 +1663,36 @@
         <v>0</v>
       </c>
       <c r="K18" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C19" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G19">
         <v>1</v>
       </c>
       <c r="H19" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I19">
         <v>0.5</v>
@@ -1701,36 +1701,36 @@
         <v>0</v>
       </c>
       <c r="K19" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L19" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B20" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G20">
         <v>1</v>
       </c>
       <c r="H20" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I20">
         <v>1</v>
@@ -1739,36 +1739,36 @@
         <v>0</v>
       </c>
       <c r="K20" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L20" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B21" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C21" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D21" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E21" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G21">
         <v>3</v>
       </c>
       <c r="H21" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I21">
         <v>0.5</v>
@@ -1777,36 +1777,36 @@
         <v>0</v>
       </c>
       <c r="K21" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L21" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B22" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C22" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E22" t="s">
+        <v>56</v>
+      </c>
+      <c r="F22" t="s">
         <v>57</v>
-      </c>
-      <c r="F22" t="s">
-        <v>58</v>
       </c>
       <c r="G22">
         <v>1</v>
       </c>
       <c r="H22" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I22">
         <v>1</v>
@@ -1815,36 +1815,36 @@
         <v>0</v>
       </c>
       <c r="K22" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L22" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B23" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C23" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D23" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E23" t="s">
+        <v>58</v>
+      </c>
+      <c r="F23" t="s">
         <v>59</v>
-      </c>
-      <c r="F23" t="s">
-        <v>60</v>
       </c>
       <c r="G23">
         <v>3</v>
       </c>
       <c r="H23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I23">
         <v>0.35</v>
@@ -1853,36 +1853,36 @@
         <v>0</v>
       </c>
       <c r="K23" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="L23" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B24" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D24" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E24" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F24" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G24">
         <v>2</v>
       </c>
       <c r="H24" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I24">
         <v>0.39</v>
@@ -1891,36 +1891,36 @@
         <v>0</v>
       </c>
       <c r="K24" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L24" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B25" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C25" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D25" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E25" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F25" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G25">
         <v>1</v>
       </c>
       <c r="H25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I25">
         <v>0.34</v>
@@ -1929,36 +1929,36 @@
         <v>0</v>
       </c>
       <c r="K25" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="L25" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B26" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C26" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D26" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E26" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F26" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G26">
         <v>1</v>
       </c>
       <c r="H26" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I26">
         <v>0.79</v>
@@ -1967,36 +1967,36 @@
         <v>0</v>
       </c>
       <c r="K26" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="L26" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B27" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C27" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D27" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E27" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G27">
         <v>2</v>
       </c>
       <c r="H27" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I27">
         <v>0.36</v>
@@ -2005,36 +2005,36 @@
         <v>0</v>
       </c>
       <c r="K27" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L27" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B28" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C28" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D28" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E28" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F28" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G28">
         <v>7</v>
       </c>
       <c r="H28" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I28">
         <v>0.4</v>
@@ -2043,36 +2043,36 @@
         <v>0</v>
       </c>
       <c r="K28" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="L28" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D29" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E29" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F29" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G29">
         <v>1</v>
       </c>
       <c r="H29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I29">
         <v>0.5</v>
@@ -2081,36 +2081,36 @@
         <v>0</v>
       </c>
       <c r="K29" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L29" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B30" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C30" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E30" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F30" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G30">
         <v>1</v>
       </c>
       <c r="H30" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I30">
         <v>1.5</v>
@@ -2119,36 +2119,36 @@
         <v>0</v>
       </c>
       <c r="K30" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L30" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C31" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D31" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E31" t="s">
+        <v>72</v>
+      </c>
+      <c r="F31" t="s">
         <v>73</v>
-      </c>
-      <c r="F31" t="s">
-        <v>74</v>
       </c>
       <c r="G31">
         <v>1</v>
       </c>
       <c r="H31" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I31">
         <v>0.45</v>
@@ -2157,36 +2157,36 @@
         <v>0</v>
       </c>
       <c r="K31" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L31" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B32" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C32" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D32" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E32" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F32" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G32">
         <v>1</v>
       </c>
       <c r="H32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I32">
         <v>0.13</v>
@@ -2195,36 +2195,36 @@
         <v>0</v>
       </c>
       <c r="K32" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L32" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B33" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C33" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D33" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E33" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F33" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G33">
         <v>1</v>
       </c>
       <c r="H33" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I33">
         <v>0.18</v>
@@ -2233,36 +2233,36 @@
         <v>0</v>
       </c>
       <c r="K33" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="L33" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B34" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C34" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D34" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E34" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F34" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G34">
         <v>1</v>
       </c>
       <c r="H34" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I34">
         <v>0.4</v>
@@ -2271,36 +2271,36 @@
         <v>0</v>
       </c>
       <c r="K34" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L34" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B35" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C35" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D35" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E35" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F35" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G35">
         <v>1</v>
       </c>
       <c r="H35" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I35">
         <v>0.28000000000000003</v>
@@ -2309,36 +2309,36 @@
         <v>0</v>
       </c>
       <c r="K35" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="L35" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B36" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C36" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D36" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E36" t="s">
+        <v>82</v>
+      </c>
+      <c r="F36" t="s">
         <v>83</v>
-      </c>
-      <c r="F36" t="s">
-        <v>84</v>
       </c>
       <c r="G36">
         <v>2</v>
       </c>
       <c r="H36" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I36">
         <v>0.2</v>
@@ -2347,36 +2347,36 @@
         <v>0</v>
       </c>
       <c r="K36" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="L36" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B37" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C37" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D37" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E37" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F37" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G37">
         <v>3</v>
       </c>
       <c r="H37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I37">
         <v>0.42</v>
@@ -2385,36 +2385,36 @@
         <v>0</v>
       </c>
       <c r="K37" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="L37" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B38" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C38" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D38" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E38" t="s">
+        <v>87</v>
+      </c>
+      <c r="F38" t="s">
         <v>88</v>
-      </c>
-      <c r="F38" t="s">
-        <v>89</v>
       </c>
       <c r="G38">
         <v>1</v>
       </c>
       <c r="H38" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I38">
         <v>0.59</v>
@@ -2423,36 +2423,36 @@
         <v>0</v>
       </c>
       <c r="K38" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L38" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B39" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C39" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D39" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E39" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F39" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G39">
         <v>1</v>
       </c>
       <c r="H39" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I39">
         <v>0.82</v>
@@ -2461,36 +2461,36 @@
         <v>0</v>
       </c>
       <c r="K39" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="L39" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B40" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C40" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D40" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E40" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F40" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G40">
         <v>2</v>
       </c>
       <c r="H40" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I40">
         <v>0.25</v>
@@ -2499,36 +2499,36 @@
         <v>0</v>
       </c>
       <c r="K40" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L40" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B41" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C41" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D41" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E41" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F41" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G41">
         <v>1</v>
       </c>
       <c r="H41" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I41">
         <v>0.28999999999999998</v>
@@ -2537,36 +2537,36 @@
         <v>0</v>
       </c>
       <c r="K41" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L41" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B42" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C42" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D42" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E42" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F42" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G42">
         <v>2</v>
       </c>
       <c r="H42" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I42">
         <v>0.19</v>
@@ -2575,36 +2575,36 @@
         <v>0</v>
       </c>
       <c r="K42" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L42" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B43" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C43" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D43" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E43" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F43" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G43">
         <v>3</v>
       </c>
       <c r="H43" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I43">
         <v>0.38</v>
@@ -2613,36 +2613,36 @@
         <v>0</v>
       </c>
       <c r="K43" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L43" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B44" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C44" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D44" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E44" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F44" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G44">
         <v>1</v>
       </c>
       <c r="H44" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I44">
         <v>0.35</v>
@@ -2651,36 +2651,36 @@
         <v>0</v>
       </c>
       <c r="K44" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L44" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B45" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C45" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D45" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E45" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F45" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G45">
         <v>2</v>
       </c>
       <c r="H45" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I45">
         <v>0.26500000000000001</v>
@@ -2689,36 +2689,36 @@
         <v>0</v>
       </c>
       <c r="K45" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L45" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B46" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C46" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D46" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E46" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F46" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G46">
         <v>1</v>
       </c>
       <c r="H46" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I46">
         <v>0.12</v>
@@ -2727,36 +2727,36 @@
         <v>0</v>
       </c>
       <c r="K46" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L46" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B47" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C47" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D47" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E47" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F47" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G47">
         <v>1</v>
       </c>
       <c r="H47" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I47">
         <v>0.43</v>
@@ -2765,36 +2765,36 @@
         <v>0</v>
       </c>
       <c r="K47" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L47" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B48" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C48" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D48" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E48" t="s">
+        <v>103</v>
+      </c>
+      <c r="F48" t="s">
         <v>104</v>
-      </c>
-      <c r="F48" t="s">
-        <v>105</v>
       </c>
       <c r="G48">
         <v>1</v>
       </c>
       <c r="H48" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I48">
         <v>0.87</v>
@@ -2803,36 +2803,36 @@
         <v>0</v>
       </c>
       <c r="K48" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="L48" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B49" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C49" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D49" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E49" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F49" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G49">
         <v>16</v>
       </c>
       <c r="H49" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I49">
         <v>0.22</v>
@@ -2841,36 +2841,36 @@
         <v>0</v>
       </c>
       <c r="K49" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L49" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B50" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C50" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D50" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E50" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F50" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G50">
         <v>1</v>
       </c>
       <c r="H50" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I50">
         <v>0.05</v>
@@ -2879,36 +2879,36 @@
         <v>0</v>
       </c>
       <c r="K50" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L50" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B51" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C51" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D51" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E51" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F51" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G51">
         <v>4</v>
       </c>
       <c r="H51" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I51">
         <v>0.44</v>
@@ -2917,36 +2917,36 @@
         <v>0</v>
       </c>
       <c r="K51" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="L51" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B52" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C52" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D52" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E52" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F52" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G52">
         <v>1</v>
       </c>
       <c r="H52" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I52">
         <v>0.2</v>
@@ -2955,36 +2955,36 @@
         <v>0</v>
       </c>
       <c r="K52" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L52" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B53" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C53" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D53" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E53" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F53" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G53">
         <v>1</v>
       </c>
       <c r="H53" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I53">
         <v>2</v>
@@ -2993,36 +2993,36 @@
         <v>0</v>
       </c>
       <c r="K53" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="L53" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B54" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C54" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D54" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E54" t="s">
+        <v>117</v>
+      </c>
+      <c r="F54" t="s">
         <v>118</v>
-      </c>
-      <c r="F54" t="s">
-        <v>119</v>
       </c>
       <c r="G54">
         <v>2</v>
       </c>
       <c r="H54" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I54">
         <v>0.22500000000000001</v>
@@ -3031,36 +3031,36 @@
         <v>0</v>
       </c>
       <c r="K54" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L54" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B55" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C55" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D55" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E55" t="s">
+        <v>119</v>
+      </c>
+      <c r="F55" t="s">
         <v>120</v>
-      </c>
-      <c r="F55" t="s">
-        <v>121</v>
       </c>
       <c r="G55">
         <v>9</v>
       </c>
       <c r="H55" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I55">
         <v>0.14399999999999999</v>
@@ -3069,36 +3069,36 @@
         <v>0</v>
       </c>
       <c r="K55" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="L55" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B56" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C56" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D56" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E56" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F56" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G56">
         <v>4</v>
       </c>
       <c r="H56" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I56">
         <v>0.2</v>
@@ -3107,36 +3107,36 @@
         <v>0</v>
       </c>
       <c r="K56" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L56" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B57" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C57" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D57" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E57" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F57" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G57">
         <v>1</v>
       </c>
       <c r="H57" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I57">
         <v>0.27</v>
@@ -3145,36 +3145,36 @@
         <v>0</v>
       </c>
       <c r="K57" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L57" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B58" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C58" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D58" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E58" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F58" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G58">
         <v>1</v>
       </c>
       <c r="H58" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I58">
         <v>0.46</v>
@@ -3183,36 +3183,36 @@
         <v>0</v>
       </c>
       <c r="K58" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="L58" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B59" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C59" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D59" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E59" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F59" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G59">
         <v>1</v>
       </c>
       <c r="H59" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I59">
         <v>0.05</v>
@@ -3221,36 +3221,36 @@
         <v>0</v>
       </c>
       <c r="K59" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="L59" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B60" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C60" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D60" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E60" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F60" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G60">
         <v>1</v>
       </c>
       <c r="H60" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I60">
         <v>0.13</v>
@@ -3259,36 +3259,36 @@
         <v>0</v>
       </c>
       <c r="K60" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="L60" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B61" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C61" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D61" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E61" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F61" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G61">
         <v>3</v>
       </c>
       <c r="H61" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I61">
         <v>0.21</v>
@@ -3297,36 +3297,36 @@
         <v>0</v>
       </c>
       <c r="K61" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="L61" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B62" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C62" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D62" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E62" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F62" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G62">
         <v>7</v>
       </c>
       <c r="H62" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I62">
         <v>0.16</v>
@@ -3335,36 +3335,36 @@
         <v>0</v>
       </c>
       <c r="K62" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="L62" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B63" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C63" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D63" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E63" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F63" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G63">
         <v>3</v>
       </c>
       <c r="H63" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I63">
         <v>4.2999999999999997E-2</v>
@@ -3373,36 +3373,36 @@
         <v>0</v>
       </c>
       <c r="K63" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="L63" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B64" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C64" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D64" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E64" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F64" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G64">
         <v>2</v>
       </c>
       <c r="H64" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I64">
         <v>0.32500000000000001</v>
@@ -3411,36 +3411,36 @@
         <v>0</v>
       </c>
       <c r="K64" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L64" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B65" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C65" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D65" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E65" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F65" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G65">
         <v>3</v>
       </c>
       <c r="H65" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I65">
         <v>0.59</v>
@@ -3449,36 +3449,36 @@
         <v>0</v>
       </c>
       <c r="K65" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="L65" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B66" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C66" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D66" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E66" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F66" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G66">
         <v>11</v>
       </c>
       <c r="H66" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I66">
         <v>0.42</v>
@@ -3487,36 +3487,36 @@
         <v>0</v>
       </c>
       <c r="K66" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L66" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B67" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C67" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D67" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E67" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F67" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G67">
         <v>1</v>
       </c>
       <c r="H67" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I67">
         <v>0.56999999999999995</v>
@@ -3525,36 +3525,36 @@
         <v>0</v>
       </c>
       <c r="K67" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L67" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B68" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C68" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D68" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E68" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F68" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G68">
         <v>2</v>
       </c>
       <c r="H68" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I68">
         <v>0.64500000000000002</v>
@@ -3563,36 +3563,36 @@
         <v>0</v>
       </c>
       <c r="K68" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L68" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B69" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C69" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D69" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E69" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F69" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G69">
         <v>2</v>
       </c>
       <c r="H69" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I69">
         <v>0.22500000000000001</v>
@@ -3601,36 +3601,36 @@
         <v>121</v>
       </c>
       <c r="K69" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="L69" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B70" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C70" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D70" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E70" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F70" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G70">
         <v>2</v>
       </c>
       <c r="H70" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I70">
         <v>7.0000000000000007E-2</v>
@@ -3639,36 +3639,36 @@
         <v>144</v>
       </c>
       <c r="K70" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="L70" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B71" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C71" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D71" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E71" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F71" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G71">
         <v>6</v>
       </c>
       <c r="H71" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I71">
         <v>0.377</v>
@@ -3677,36 +3677,36 @@
         <v>75.83</v>
       </c>
       <c r="K71" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L71" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B72" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C72" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D72" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E72" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F72" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G72">
         <v>1</v>
       </c>
       <c r="H72" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I72">
         <v>0.25</v>
@@ -3715,36 +3715,36 @@
         <v>499</v>
       </c>
       <c r="K72" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="L72" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B73" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C73" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D73" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E73" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F73" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G73">
         <v>1</v>
       </c>
       <c r="H73" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I73">
         <v>0.25</v>
@@ -3753,36 +3753,36 @@
         <v>499</v>
       </c>
       <c r="K73" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="L73" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B74" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C74" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D74" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E74" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F74" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G74">
         <v>11</v>
       </c>
       <c r="H74" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I74">
         <v>0.35</v>
@@ -3791,36 +3791,36 @@
         <v>59</v>
       </c>
       <c r="K74" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L74" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B75" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C75" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D75" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E75" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F75" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G75">
         <v>3</v>
       </c>
       <c r="H75" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I75">
         <v>0.4</v>
@@ -3829,36 +3829,36 @@
         <v>84</v>
       </c>
       <c r="K75" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L75" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B76" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C76" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D76" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E76" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F76" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G76">
         <v>1</v>
       </c>
       <c r="H76" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I76">
         <v>0.44</v>
@@ -3867,36 +3867,36 @@
         <v>84</v>
       </c>
       <c r="K76" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="L76" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B77" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C77" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D77" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E77" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F77" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G77">
         <v>1</v>
       </c>
       <c r="H77" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I77">
         <v>0.31</v>
@@ -3905,36 +3905,36 @@
         <v>149</v>
       </c>
       <c r="K77" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L77" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B78" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C78" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D78" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E78" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F78" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G78">
         <v>3</v>
       </c>
       <c r="H78" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I78">
         <v>0.433</v>
@@ -3943,36 +3943,36 @@
         <v>198</v>
       </c>
       <c r="K78" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="L78" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B79" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C79" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D79" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E79" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F79" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G79">
         <v>3</v>
       </c>
       <c r="H79" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I79">
         <v>10</v>
@@ -3981,36 +3981,36 @@
         <v>0</v>
       </c>
       <c r="K79" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L79" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B80" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C80" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D80" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E80" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F80" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G80">
         <v>1</v>
       </c>
       <c r="H80" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I80">
         <v>0.53</v>
@@ -4019,36 +4019,36 @@
         <v>227</v>
       </c>
       <c r="K80" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L80" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B81" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C81" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D81" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E81" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F81" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G81">
         <v>2</v>
       </c>
       <c r="H81" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I81">
         <v>0.18</v>
@@ -4057,36 +4057,36 @@
         <v>35.200000000000003</v>
       </c>
       <c r="K81" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="L81" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B82" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C82" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D82" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E82" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F82" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G82">
         <v>3</v>
       </c>
       <c r="H82" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I82">
         <v>0.38300000000000001</v>
@@ -4095,36 +4095,36 @@
         <v>55</v>
       </c>
       <c r="K82" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L82" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="83" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B83" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C83" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D83" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E83" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F83" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G83">
         <v>2</v>
       </c>
       <c r="H83" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I83">
         <v>0.13</v>
@@ -4133,36 +4133,36 @@
         <v>35</v>
       </c>
       <c r="K83" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="L83" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B84" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C84" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D84" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E84" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F84" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G84">
         <v>7</v>
       </c>
       <c r="H84" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I84">
         <v>0.45</v>
@@ -4171,36 +4171,36 @@
         <v>45.5</v>
       </c>
       <c r="K84" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L84" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="85" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
+        <v>169</v>
+      </c>
+      <c r="B85" t="s">
+        <v>11</v>
+      </c>
+      <c r="C85" t="s">
         <v>170</v>
       </c>
-      <c r="B85" t="s">
-        <v>12</v>
-      </c>
-      <c r="C85" t="s">
+      <c r="D85" t="s">
+        <v>13</v>
+      </c>
+      <c r="E85" t="s">
         <v>171</v>
       </c>
-      <c r="D85" t="s">
-        <v>14</v>
-      </c>
-      <c r="E85" t="s">
-        <v>172</v>
-      </c>
       <c r="F85" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G85">
         <v>8352</v>
       </c>
       <c r="H85" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I85">
         <v>0.18</v>
@@ -4209,36 +4209,36 @@
         <v>0</v>
       </c>
       <c r="K85" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L85" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="86" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
+        <v>169</v>
+      </c>
+      <c r="B86" t="s">
+        <v>11</v>
+      </c>
+      <c r="C86" t="s">
         <v>170</v>
       </c>
-      <c r="B86" t="s">
-        <v>12</v>
-      </c>
-      <c r="C86" t="s">
-        <v>171</v>
-      </c>
       <c r="D86" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E86" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F86" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G86">
         <v>21</v>
       </c>
       <c r="H86" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I86">
         <v>0.56999999999999995</v>
@@ -4247,36 +4247,36 @@
         <v>316</v>
       </c>
       <c r="K86" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L86" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="87" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
+        <v>169</v>
+      </c>
+      <c r="B87" t="s">
+        <v>11</v>
+      </c>
+      <c r="C87" t="s">
         <v>170</v>
       </c>
-      <c r="B87" t="s">
-        <v>12</v>
-      </c>
-      <c r="C87" t="s">
-        <v>171</v>
-      </c>
       <c r="D87" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E87" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F87" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G87">
         <v>27</v>
       </c>
       <c r="H87" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I87">
         <v>0.33</v>
@@ -4285,36 +4285,36 @@
         <v>111</v>
       </c>
       <c r="K87" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L87" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="88" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
+        <v>169</v>
+      </c>
+      <c r="B88" t="s">
+        <v>11</v>
+      </c>
+      <c r="C88" t="s">
         <v>170</v>
       </c>
-      <c r="B88" t="s">
-        <v>12</v>
-      </c>
-      <c r="C88" t="s">
-        <v>171</v>
-      </c>
       <c r="D88" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E88" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F88" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G88">
         <v>12</v>
       </c>
       <c r="H88" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I88">
         <v>0.86</v>
@@ -4323,10 +4323,10 @@
         <v>91</v>
       </c>
       <c r="K88" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="L88" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>